<commit_message>
Complete AI business anomaly monitoring system
</commit_message>
<xml_diff>
--- a/data/business_metrics.xlsx
+++ b/data/business_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\siddh\OneDrive\Desktop\AI Bussiness Anamoly Monitor\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24BC7D9D-925C-408B-BE0F-8118538D3D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51634FAA-F1EF-4C36-A3C3-34654C2CC497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -998,6 +998,29 @@
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A22" s="4">
+        <v>46243</v>
+      </c>
+      <c r="B22" s="2">
+        <v>150000</v>
+      </c>
+      <c r="C22" s="2">
+        <v>1620</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E22" s="2">
+        <v>65000</v>
+      </c>
+      <c r="F22" s="2">
+        <v>32000</v>
+      </c>
+      <c r="G22" s="2">
+        <v>6000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>